<commit_message>
Check-up fixes: Bhutan placeholder 99999.999 / negatives / upper-bound flags; PGCB demand keying slip; Sri Lanka unpublished zero days removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjcnPNGA6ZkWeQkXXc23hq
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/bhutan_power_generation_daily.xlsx
+++ b/output/Data and Chart Outputs/bhutan_power_generation_daily.xlsx
@@ -973,7 +973,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Flags: values blanked because they fall below 30% of the centred 15-day median of their series - BPSO's daily sheets carry occasional keying slips (e.g. 8,200 for 82,000 MWh).</t>
+          <t>Flags: values blanked because they fall below 30% (generation, energy met, peak: or above 4x) the centred 15-day median of their series - BPSO's daily sheets carry occasional keying slips (e.g. 8,200 for 82,000 MWh). BPSO's placeholder 99999.999 and negative energy values are blanked too (not listed).</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
         <v>46204</v>
       </c>
       <c r="B38" t="n">
-        <v>2405.468569</v>
+        <v>2305.46857</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -4734,9 +4734,6 @@
       <c r="D100" t="n">
         <v>17830</v>
       </c>
-      <c r="E100" t="n">
-        <v>99999.999</v>
-      </c>
       <c r="F100" t="n">
         <v>0</v>
       </c>
@@ -5290,6 +5287,9 @@
       <c r="D123" t="n">
         <v>17480</v>
       </c>
+      <c r="E123" t="n">
+        <v>387.4</v>
+      </c>
       <c r="F123" t="n">
         <v>0</v>
       </c>
@@ -5414,9 +5414,6 @@
       <c r="D128" t="n">
         <v>19816</v>
       </c>
-      <c r="E128" t="n">
-        <v>99999.999</v>
-      </c>
       <c r="F128" t="n">
         <v>0</v>
       </c>
@@ -5469,9 +5466,6 @@
       <c r="E130" t="n">
         <v>0</v>
       </c>
-      <c r="F130" t="n">
-        <v>-1131.865</v>
-      </c>
       <c r="G130" t="n">
         <v>860</v>
       </c>
@@ -5547,9 +5541,6 @@
       <c r="E133" t="n">
         <v>0</v>
       </c>
-      <c r="F133" t="n">
-        <v>-2540</v>
-      </c>
       <c r="G133" t="n">
         <v>0</v>
       </c>
@@ -5573,9 +5564,6 @@
       <c r="E134" t="n">
         <v>0</v>
       </c>
-      <c r="F134" t="n">
-        <v>-2710</v>
-      </c>
       <c r="G134" t="n">
         <v>0</v>
       </c>
@@ -5651,9 +5639,6 @@
       <c r="E137" t="n">
         <v>0</v>
       </c>
-      <c r="F137" t="n">
-        <v>-2565.588</v>
-      </c>
       <c r="G137" t="n">
         <v>0</v>
       </c>
@@ -5781,9 +5766,6 @@
       <c r="E142" t="n">
         <v>0</v>
       </c>
-      <c r="F142" t="n">
-        <v>-3226.183</v>
-      </c>
       <c r="G142" t="n">
         <v>0</v>
       </c>
@@ -5859,9 +5841,6 @@
       <c r="E145" t="n">
         <v>0</v>
       </c>
-      <c r="F145" t="n">
-        <v>-3830.61</v>
-      </c>
       <c r="G145" t="n">
         <v>0</v>
       </c>
@@ -5885,9 +5864,6 @@
       <c r="E146" t="n">
         <v>0</v>
       </c>
-      <c r="F146" t="n">
-        <v>-4843.455</v>
-      </c>
       <c r="G146" t="n">
         <v>0</v>
       </c>
@@ -8797,9 +8773,6 @@
       <c r="G258" t="n">
         <v>0</v>
       </c>
-      <c r="H258" t="n">
-        <v>-2182.332</v>
-      </c>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n">
@@ -24518,9 +24491,6 @@
       <c r="C866" t="n">
         <v>87962</v>
       </c>
-      <c r="D866" t="n">
-        <v>99999.999</v>
-      </c>
       <c r="E866" t="n">
         <v>49659</v>
       </c>
@@ -24615,12 +24585,6 @@
     <row r="870">
       <c r="A870" s="4" t="n">
         <v>46210</v>
-      </c>
-      <c r="B870" t="n">
-        <v>99999.999</v>
-      </c>
-      <c r="C870" t="n">
-        <v>99999.999</v>
       </c>
       <c r="D870" t="n">
         <v>35065.76</v>
@@ -34224,7 +34188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34614,7 +34578,7 @@
         <v>21.17</v>
       </c>
       <c r="D24" t="n">
-        <v>18413.6</v>
+        <v>17645.3</v>
       </c>
     </row>
     <row r="25">
@@ -34630,7 +34594,7 @@
         <v>14.195</v>
       </c>
       <c r="D25" t="n">
-        <v>11360</v>
+        <v>10243.9</v>
       </c>
     </row>
     <row r="26">
@@ -34715,7 +34679,7 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>45237</v>
+        <v>45239</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -34723,15 +34687,15 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>387.4</v>
+        <v>234</v>
       </c>
       <c r="D31" t="n">
-        <v>1800</v>
+        <v>1183.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>45239</v>
+        <v>45444</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -34739,15 +34703,15 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>1800</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>45444</v>
+        <v>45445</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -34763,7 +34727,7 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>45445</v>
+        <v>45454</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -34771,15 +34735,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>1644</v>
       </c>
       <c r="D34" t="n">
-        <v>2360</v>
+        <v>6088</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>45454</v>
+        <v>45623</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -34787,15 +34751,15 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1644</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>6088</v>
+        <v>508</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>45623</v>
+        <v>46012</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -34806,12 +34770,12 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>508</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>46012</v>
+        <v>46019</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -34822,12 +34786,12 @@
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>74</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>46019</v>
+        <v>46023</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -34838,12 +34802,12 @@
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>46023</v>
+        <v>46024</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -34854,12 +34818,12 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>46024</v>
+        <v>46033</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -34870,12 +34834,12 @@
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>46033</v>
+        <v>46044</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -34886,12 +34850,12 @@
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>150</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>46044</v>
+        <v>46045</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -34902,12 +34866,12 @@
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>46045</v>
+        <v>46046</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -34918,12 +34882,12 @@
         <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>150</v>
+        <v>187</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>46046</v>
+        <v>46047</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -34939,7 +34903,7 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>46047</v>
+        <v>46048</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -34947,7 +34911,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>0.051</v>
       </c>
       <c r="D45" t="n">
         <v>187</v>
@@ -34955,7 +34919,7 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>46048</v>
+        <v>46078</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -34963,15 +34927,15 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.051</v>
+        <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>187</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -34982,12 +34946,12 @@
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
-        <v>46079</v>
+        <v>46081</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -34998,12 +34962,12 @@
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>75</v>
+        <v>203</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -35014,12 +34978,12 @@
         <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>203</v>
+        <v>310.1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
-        <v>46082</v>
+        <v>46149</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -35027,15 +34991,15 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="D50" t="n">
-        <v>310.1</v>
+        <v>798</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -35043,15 +35007,15 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>798</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -35062,12 +35026,12 @@
         <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>1130</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -35075,15 +35039,15 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="D53" t="n">
-        <v>1193</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
-        <v>46152</v>
+        <v>46154</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -35091,15 +35055,15 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>520</v>
+        <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>1754</v>
+        <v>3970</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
-        <v>46154</v>
+        <v>46174</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -35107,15 +35071,15 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>4196</v>
       </c>
       <c r="D55" t="n">
-        <v>3970</v>
+        <v>14298</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -35123,15 +35087,15 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4196</v>
+        <v>6.477</v>
       </c>
       <c r="D56" t="n">
-        <v>14298</v>
+        <v>13809</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
-        <v>46175</v>
+        <v>46258</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -35139,25 +35103,9 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6.477</v>
+        <v>53.046</v>
       </c>
       <c r="D57" t="n">
-        <v>13809</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Exports_MWh</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>53.046</v>
-      </c>
-      <c r="D58" t="n">
         <v>49326</v>
       </c>
     </row>

</xml_diff>